<commit_message>
Add as-of date stamps, quarterly refresh process, hyperlinked Tableau sources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013tgD7fbckVrxCtXTJMuFAX
</commit_message>
<xml_diff>
--- a/workbook/IP_Distribution_Cost_Variance_Model.xlsx
+++ b/workbook/IP_Distribution_Cost_Variance_Model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="254">
   <si>
     <t xml:space="preserve">IP Distribution Decision Verticals: Cost Variance Model</t>
   </si>
@@ -35,6 +35,9 @@
     <t xml:space="preserve">Edit inputs on the Assumptions sheet. Everything on this page recalculates.</t>
   </si>
   <si>
+    <t xml:space="preserve">Prices, fees and rates as of October 11, 2026. Refreshed quarterly; next refresh January 11, 2027.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Platform</t>
   </si>
   <si>
@@ -785,7 +788,7 @@
     <t xml:space="preserve">https://scribecount.com/tools/platform-comparison</t>
   </si>
   <si>
-    <t xml:space="preserve">Fees change often. Figures reflect sources available as of October 2026. Not legal or financial advice.</t>
+    <t xml:space="preserve">Fees change often. Figures are as of October 11, 2026 and are refreshed quarterly. Not legal or financial advice.</t>
   </si>
 </sst>
 </file>
@@ -805,7 +808,7 @@
     <numFmt numFmtId="173" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="174" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -853,6 +856,14 @@
       <i val="true"/>
       <sz val="11"/>
       <color rgb="FF595959"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1003,7 +1014,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1028,35 +1039,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1064,51 +1079,59 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1116,31 +1139,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1148,11 +1163,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1169,7 +1184,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1381,11 +1396,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="15605282"/>
-        <c:axId val="71512213"/>
+        <c:axId val="53472724"/>
+        <c:axId val="53561847"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="15605282"/>
+        <c:axId val="53472724"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1417,7 +1432,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71512213"/>
+        <c:crossAx val="53561847"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1425,7 +1440,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71512213"/>
+        <c:axId val="53561847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1501,7 +1516,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15605282"/>
+        <c:crossAx val="53472724"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1688,11 +1703,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65481837"/>
-        <c:axId val="58096159"/>
+        <c:axId val="14274948"/>
+        <c:axId val="83975191"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65481837"/>
+        <c:axId val="14274948"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1724,7 +1739,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58096159"/>
+        <c:crossAx val="83975191"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1732,7 +1747,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58096159"/>
+        <c:axId val="83975191"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1808,7 +1823,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65481837"/>
+        <c:crossAx val="14274948"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1995,11 +2010,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="53119984"/>
-        <c:axId val="10054524"/>
+        <c:axId val="35356178"/>
+        <c:axId val="58806989"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="53119984"/>
+        <c:axId val="35356178"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2031,7 +2046,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10054524"/>
+        <c:crossAx val="58806989"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2039,7 +2054,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="10054524"/>
+        <c:axId val="58806989"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2115,7 +2130,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53119984"/>
+        <c:crossAx val="35356178"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2154,9 +2169,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>65160</xdr:colOff>
+      <xdr:colOff>64800</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>152280</xdr:rowOff>
+      <xdr:rowOff>151920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2165,7 +2180,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="5159880"/>
-        <a:ext cx="6479280" cy="2879280"/>
+        <a:ext cx="6478920" cy="2878920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2189,9 +2204,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>261720</xdr:colOff>
+      <xdr:colOff>261360</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>182520</xdr:rowOff>
+      <xdr:rowOff>182160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2200,7 +2215,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="1832760" y="3827520"/>
-        <a:ext cx="5759280" cy="2879640"/>
+        <a:ext cx="5758920" cy="2879280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2224,9 +2239,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>543240</xdr:colOff>
+      <xdr:colOff>542880</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>182520</xdr:rowOff>
+      <xdr:rowOff>182160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2235,7 +2250,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="1973520" y="3637080"/>
-        <a:ext cx="5759280" cy="2879640"/>
+        <a:ext cx="5758920" cy="2879280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2482,7 +2497,9 @@
       <c r="I3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3"/>
+      <c r="A4" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -2493,250 +2510,250 @@
       <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>10</v>
       </c>
+      <c r="I5" s="7" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="8" t="n">
+      <c r="A6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="9" t="n">
         <f aca="false">'Monthly Scenario'!D5</f>
         <v>6.794</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!B5,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>0</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <f aca="false">'Monthly Scenario'!E5</f>
         <v>3.283</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="9" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!C5,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>0</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <f aca="false">'Fixed Costs'!J5</f>
         <v>0</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="9" t="n">
         <f aca="false">'Monthly Scenario'!M5</f>
         <v>6046.2</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="9" t="n">
         <f aca="false">'Monthly Scenario'!N5</f>
         <v>0</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="10" t="n">
         <f aca="false">'Monthly Scenario'!O5</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="8" t="n">
+      <c r="A7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="9" t="n">
         <f aca="false">'Monthly Scenario'!D6</f>
         <v>3.3269375</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!B6,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>-3.4670625</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <f aca="false">'Monthly Scenario'!E6</f>
         <v>2.96905</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!C6,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>-0.31395</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <f aca="false">'Fixed Costs'!J6</f>
         <v>125</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="9" t="n">
         <f aca="false">'Monthly Scenario'!M6</f>
         <v>3652.5925</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="9" t="n">
         <f aca="false">'Monthly Scenario'!N6</f>
         <v>-2393.6075</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I7" s="10" t="n">
         <f aca="false">'Monthly Scenario'!O6</f>
         <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="8" t="n">
+      <c r="A8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="9" t="n">
         <f aca="false">'Monthly Scenario'!D7</f>
         <v>5.8445</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="9" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!B7,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>-0.949499999999999</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <f aca="false">'Monthly Scenario'!E7</f>
         <v>3.493</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!C7,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>0.21</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <f aca="false">'Fixed Costs'!J7</f>
         <v>20</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="9" t="n">
         <f aca="false">'Monthly Scenario'!M7</f>
         <v>5477.5</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="9" t="n">
         <f aca="false">'Monthly Scenario'!N7</f>
         <v>-568.699999999999</v>
       </c>
-      <c r="I8" s="9" t="n">
+      <c r="I8" s="10" t="n">
         <f aca="false">'Monthly Scenario'!O7</f>
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="8" t="n">
+      <c r="A9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="9" t="n">
         <f aca="false">'Monthly Scenario'!D8</f>
         <v>2.796</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="9" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!B8,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>-3.998</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <f aca="false">'Monthly Scenario'!E8</f>
         <v>1.996</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!C8,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>-1.287</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <f aca="false">'Fixed Costs'!J8</f>
         <v>125</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <f aca="false">'Monthly Scenario'!M8</f>
         <v>2863.2</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="9" t="n">
         <f aca="false">'Monthly Scenario'!N8</f>
         <v>-3183</v>
       </c>
-      <c r="I9" s="9" t="n">
+      <c r="I9" s="10" t="n">
         <f aca="false">'Monthly Scenario'!O8</f>
         <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="8" t="n">
+      <c r="A10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="9" t="n">
         <f aca="false">'Monthly Scenario'!D9</f>
         <v>3.6455</v>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="9" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!B9,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>-3.1485</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="9" t="n">
         <f aca="false">'Monthly Scenario'!E9</f>
         <v>3.493</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="9" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!C9,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>0.21</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="9" t="n">
         <f aca="false">'Fixed Costs'!J9</f>
         <v>12</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="9" t="n">
         <f aca="false">'Monthly Scenario'!M9</f>
         <v>3990.22</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="9" t="n">
         <f aca="false">'Monthly Scenario'!N9</f>
         <v>-2055.98</v>
       </c>
-      <c r="I10" s="9" t="n">
+      <c r="I10" s="10" t="n">
         <f aca="false">'Monthly Scenario'!O9</f>
         <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="8" t="n">
+      <c r="B11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="9" t="n">
         <f aca="false">'Monthly Scenario'!E10</f>
         <v>3.1437</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="9" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$I$5:$I$11,MATCH('Monthly Scenario'!C10,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>-0.1393</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="9" t="n">
         <f aca="false">'Fixed Costs'!J10</f>
         <v>292.88</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="9" t="n">
         <f aca="false">'Monthly Scenario'!M10</f>
         <v>1866.22</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="9" t="n">
         <f aca="false">'Monthly Scenario'!N10</f>
         <v>-4179.98</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I11" s="10" t="n">
         <f aca="false">'Monthly Scenario'!O10</f>
         <v>6</v>
       </c>
@@ -2753,8 +2770,8 @@
       <c r="I12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>18</v>
+      <c r="A13" s="11" t="s">
+        <v>19</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -2766,82 +2783,82 @@
       <c r="I13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
+      <c r="A14" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
+      <c r="A15" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
+      <c r="A16" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
+      <c r="A17" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
+      <c r="A18" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
+      <c r="A19" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2878,8 +2895,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>25</v>
+      <c r="A1" s="13" t="s">
+        <v>26</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2887,7 +2904,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2900,543 +2917,543 @@
       <c r="D3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>30</v>
       </c>
+      <c r="D4" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
+      <c r="A5" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="16" t="n">
+      <c r="A6" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="17" t="n">
         <v>16.99</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="17" t="s">
+      <c r="C6" s="16" t="s">
         <v>34</v>
       </c>
+      <c r="D6" s="18" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="18" t="n">
+      <c r="A7" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="19" t="n">
         <v>200</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="17" t="s">
+      <c r="C7" s="16" t="s">
         <v>37</v>
       </c>
+      <c r="D7" s="18" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="16" t="n">
+      <c r="A8" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="17" t="n">
         <v>4.99</v>
       </c>
-      <c r="C8" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>39</v>
+      <c r="C8" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="19" t="n">
+      <c r="A9" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="17" t="s">
+      <c r="C9" s="16" t="s">
         <v>42</v>
       </c>
+      <c r="D9" s="18" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="18" t="n">
+      <c r="A10" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="19" t="n">
         <v>50</v>
       </c>
-      <c r="C10" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="17" t="s">
+      <c r="C10" s="16" t="s">
         <v>45</v>
       </c>
+      <c r="D10" s="18" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>50</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="18" t="n">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="16" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>52</v>
+      <c r="D14" s="18" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="17" t="s">
+      <c r="A15" s="16" t="s">
         <v>54</v>
       </c>
+      <c r="B15" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
+      <c r="A16" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" s="20" t="n">
+      <c r="A17" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="21" t="n">
         <v>0.6</v>
       </c>
-      <c r="C17" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="17" t="s">
+      <c r="C17" s="16" t="s">
         <v>57</v>
       </c>
+      <c r="D17" s="18" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" s="20" t="n">
+      <c r="A18" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="C18" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>59</v>
+      <c r="C18" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="21" t="n">
+      <c r="A19" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="22" t="n">
         <v>2.3</v>
       </c>
-      <c r="C19" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>61</v>
+      <c r="C19" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="16" t="n">
+      <c r="A20" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D20" s="17" t="s">
-        <v>63</v>
+      <c r="C20" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B21" s="21" t="n">
+      <c r="A21" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="22" t="n">
         <v>0.012</v>
       </c>
-      <c r="C21" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="17" t="s">
+      <c r="C21" s="16" t="s">
         <v>66</v>
       </c>
+      <c r="D21" s="18" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="20" t="n">
+      <c r="A22" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" s="21" t="n">
         <v>0.7</v>
       </c>
-      <c r="C22" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="17" t="s">
-        <v>68</v>
+      <c r="C22" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="20" t="n">
+      <c r="A23" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="21" t="n">
         <v>0.35</v>
       </c>
-      <c r="C23" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>70</v>
+      <c r="C23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B24" s="21" t="n">
+      <c r="A24" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="C24" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D24" s="17" t="s">
+      <c r="C24" s="16" t="s">
         <v>73</v>
       </c>
+      <c r="D24" s="18" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="24" t="n">
+        <v>0.01875</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B28" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" s="17" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B36" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B37" s="21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B39" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B40" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B42" s="25" t="n">
+        <v>125</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B43" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="C43" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B44" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B26" s="22" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="23" t="n">
-        <v>0.01875</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B28" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D28" s="17" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="D29" s="17" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="B31" s="20" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D31" s="17" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="B32" s="16" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B33" s="20" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D33" s="17" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="B35" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D35" s="17" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="B36" s="20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="D36" s="17" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="B37" s="20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="D37" s="17" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="B39" s="20" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C39" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D39" s="17" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="B40" s="20" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C40" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D40" s="17" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="B42" s="24" t="n">
-        <v>125</v>
-      </c>
-      <c r="C42" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D42" s="17" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="B43" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="C43" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D43" s="17" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="B44" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="C44" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D44" s="17" t="s">
-        <v>109</v>
+      <c r="C44" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="B45" s="16" t="n">
+      <c r="A45" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B45" s="17" t="n">
         <v>13.99</v>
       </c>
-      <c r="C45" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="D45" s="17" t="s">
+      <c r="C45" s="16" t="s">
         <v>112</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -3488,8 +3505,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>113</v>
+      <c r="A1" s="13" t="s">
+        <v>114</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3541,437 +3558,437 @@
       <c r="N3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="I4" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="J4" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="K4" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="L4" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="N4" s="6" t="s">
-        <v>10</v>
+      <c r="M4" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="C5" s="27" t="n">
+      <c r="A5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="28" t="n">
         <f aca="false">Assumptions!$B$6</f>
         <v>16.99</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="29" t="n">
         <f aca="false">Assumptions!$B$6*(1-Assumptions!$B$17)</f>
         <v>6.796</v>
       </c>
-      <c r="E5" s="28" t="n">
+      <c r="E5" s="29" t="n">
         <f aca="false">IF(Assumptions!$B$7&lt;=108,Assumptions!$B$19,Assumptions!$B$20+Assumptions!$B$7*Assumptions!$B$21)</f>
         <v>3.4</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G5" s="29" t="n">
+      <c r="G5" s="30" t="n">
         <f aca="false">C5-D5-E5-F5</f>
         <v>6.794</v>
       </c>
-      <c r="H5" s="30" t="n">
+      <c r="H5" s="31" t="n">
         <f aca="false">IFERROR(G5/C5,0)</f>
         <v>0.399882283696292</v>
       </c>
-      <c r="I5" s="28" t="n">
+      <c r="I5" s="29" t="n">
         <f aca="false">G5-INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))</f>
         <v>0</v>
       </c>
-      <c r="J5" s="30" t="n">
+      <c r="J5" s="31" t="n">
         <f aca="false">IFERROR(I5/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))),0)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="28" t="n">
+      <c r="K5" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-D5</f>
         <v>0</v>
       </c>
-      <c r="L5" s="28" t="n">
+      <c r="L5" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-E5</f>
         <v>0</v>
       </c>
-      <c r="M5" s="28" t="n">
+      <c r="M5" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-F5</f>
         <v>0</v>
       </c>
-      <c r="N5" s="26" t="n">
+      <c r="N5" s="27" t="n">
         <f aca="false">RANK(G5,$G$5:$G$11)</f>
         <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="26" t="s">
+      <c r="A6" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="B6" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="28" t="n">
         <f aca="false">Assumptions!$B$6</f>
         <v>16.99</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="29" t="n">
         <f aca="false">Assumptions!$B$6*(1-Assumptions!$B$18)</f>
         <v>10.194</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="29" t="n">
         <f aca="false">IF(Assumptions!$B$7&lt;=108,Assumptions!$B$19,Assumptions!$B$20+Assumptions!$B$7*Assumptions!$B$21)</f>
         <v>3.4</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G6" s="29" t="n">
+      <c r="G6" s="30" t="n">
         <f aca="false">C6-D6-E6-F6</f>
         <v>3.396</v>
       </c>
-      <c r="H6" s="30" t="n">
+      <c r="H6" s="31" t="n">
         <f aca="false">IFERROR(G6/C6,0)</f>
         <v>0.199882283696292</v>
       </c>
-      <c r="I6" s="28" t="n">
+      <c r="I6" s="29" t="n">
         <f aca="false">G6-INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))</f>
         <v>-3.398</v>
       </c>
-      <c r="J6" s="30" t="n">
+      <c r="J6" s="31" t="n">
         <f aca="false">IFERROR(I6/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))),0)</f>
         <v>-0.500147188695908</v>
       </c>
-      <c r="K6" s="28" t="n">
+      <c r="K6" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-D6</f>
         <v>-3.398</v>
       </c>
-      <c r="L6" s="28" t="n">
+      <c r="L6" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-E6</f>
         <v>0</v>
       </c>
-      <c r="M6" s="28" t="n">
+      <c r="M6" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-F6</f>
         <v>0</v>
       </c>
-      <c r="N6" s="26" t="n">
+      <c r="N6" s="27" t="n">
         <f aca="false">RANK(G6,$G$5:$G$11)</f>
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="C7" s="27" t="n">
+      <c r="A7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" s="28" t="n">
         <f aca="false">Assumptions!$B$6</f>
         <v>16.99</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="D7" s="29" t="n">
         <f aca="false">Assumptions!$B$6*Assumptions!$B$26</f>
         <v>9.3445</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="29" t="n">
         <f aca="false">Assumptions!$B$28</f>
         <v>4</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="29" t="n">
         <f aca="false">Assumptions!$B$6*Assumptions!$B$27</f>
         <v>0.3185625</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="30" t="n">
         <f aca="false">C7-D7-E7-F7</f>
         <v>3.3269375</v>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="31" t="n">
         <f aca="false">IFERROR(G7/C7,0)</f>
         <v>0.195817392583873</v>
       </c>
-      <c r="I7" s="28" t="n">
+      <c r="I7" s="29" t="n">
         <f aca="false">G7-INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))</f>
         <v>-3.4670625</v>
       </c>
-      <c r="J7" s="30" t="n">
+      <c r="J7" s="31" t="n">
         <f aca="false">IFERROR(I7/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))),0)</f>
         <v>-0.510312408007065</v>
       </c>
-      <c r="K7" s="28" t="n">
+      <c r="K7" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-D7</f>
         <v>-2.5485</v>
       </c>
-      <c r="L7" s="28" t="n">
+      <c r="L7" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-E7</f>
         <v>-0.6</v>
       </c>
-      <c r="M7" s="28" t="n">
+      <c r="M7" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-F7</f>
         <v>-0.3185625</v>
       </c>
-      <c r="N7" s="26" t="n">
+      <c r="N7" s="27" t="n">
         <f aca="false">RANK(G7,$G$5:$G$11)</f>
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="C8" s="27" t="n">
+      <c r="A8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" s="28" t="n">
         <f aca="false">Assumptions!$B$6</f>
         <v>16.99</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="29" t="n">
         <f aca="false">Assumptions!$B$6*(1-Assumptions!$B$31)</f>
         <v>7.6455</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="29" t="n">
         <f aca="false">Assumptions!$B$32</f>
         <v>3.5</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G8" s="29" t="n">
+      <c r="G8" s="30" t="n">
         <f aca="false">C8-D8-E8-F8</f>
         <v>5.8445</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="31" t="n">
         <f aca="false">IFERROR(G8/C8,0)</f>
         <v>0.343996468510889</v>
       </c>
-      <c r="I8" s="28" t="n">
+      <c r="I8" s="29" t="n">
         <f aca="false">G8-INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))</f>
         <v>-0.949499999999999</v>
       </c>
-      <c r="J8" s="30" t="n">
+      <c r="J8" s="31" t="n">
         <f aca="false">IFERROR(I8/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))),0)</f>
         <v>-0.139755666764792</v>
       </c>
-      <c r="K8" s="28" t="n">
+      <c r="K8" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-D8</f>
         <v>-0.849499999999999</v>
       </c>
-      <c r="L8" s="28" t="n">
+      <c r="L8" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-E8</f>
         <v>-0.1</v>
       </c>
-      <c r="M8" s="28" t="n">
+      <c r="M8" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-F8</f>
         <v>0</v>
       </c>
-      <c r="N8" s="26" t="n">
+      <c r="N8" s="27" t="n">
         <f aca="false">RANK(G8,$G$5:$G$11)</f>
         <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="B9" s="26" t="s">
+      <c r="A9" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="B9" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="C9" s="28" t="n">
         <f aca="false">Assumptions!$B$6</f>
         <v>16.99</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="29" t="n">
         <f aca="false">Assumptions!$B$35</f>
         <v>5</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="29" t="n">
         <f aca="false">(C9-D9-E9)*Assumptions!$B$37</f>
         <v>2.398</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="30" t="n">
         <f aca="false">C9-D9-E9-F9</f>
         <v>9.592</v>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="H9" s="31" t="n">
         <f aca="false">IFERROR(G9/C9,0)</f>
         <v>0.564567392583873</v>
       </c>
-      <c r="I9" s="28" t="n">
+      <c r="I9" s="29" t="n">
         <f aca="false">G9-INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))</f>
         <v>2.798</v>
       </c>
-      <c r="J9" s="30" t="n">
+      <c r="J9" s="31" t="n">
         <f aca="false">IFERROR(I9/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))),0)</f>
         <v>0.411833971151016</v>
       </c>
-      <c r="K9" s="28" t="n">
+      <c r="K9" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-D9</f>
         <v>6.796</v>
       </c>
-      <c r="L9" s="28" t="n">
+      <c r="L9" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-E9</f>
         <v>-1.6</v>
       </c>
-      <c r="M9" s="28" t="n">
+      <c r="M9" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-F9</f>
         <v>-2.398</v>
       </c>
-      <c r="N9" s="26" t="n">
+      <c r="N9" s="27" t="n">
         <f aca="false">RANK(G9,$G$5:$G$11)</f>
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="B10" s="26" t="s">
+      <c r="A10" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="B10" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="C10" s="28" t="n">
         <f aca="false">Assumptions!$B$6</f>
         <v>16.99</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="29" t="n">
         <f aca="false">Assumptions!$B$6*Assumptions!$B$36</f>
         <v>8.495</v>
       </c>
-      <c r="E10" s="28" t="n">
+      <c r="E10" s="29" t="n">
         <f aca="false">Assumptions!$B$35</f>
         <v>5</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="29" t="n">
         <f aca="false">(C10-D10-E10)*Assumptions!$B$37</f>
         <v>0.699</v>
       </c>
-      <c r="G10" s="29" t="n">
+      <c r="G10" s="30" t="n">
         <f aca="false">C10-D10-E10-F10</f>
         <v>2.796</v>
       </c>
-      <c r="H10" s="30" t="n">
+      <c r="H10" s="31" t="n">
         <f aca="false">IFERROR(G10/C10,0)</f>
         <v>0.164567392583873</v>
       </c>
-      <c r="I10" s="28" t="n">
+      <c r="I10" s="29" t="n">
         <f aca="false">G10-INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))</f>
         <v>-3.998</v>
       </c>
-      <c r="J10" s="30" t="n">
+      <c r="J10" s="31" t="n">
         <f aca="false">IFERROR(I10/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))),0)</f>
         <v>-0.588460406240801</v>
       </c>
-      <c r="K10" s="28" t="n">
+      <c r="K10" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-D10</f>
         <v>-1.699</v>
       </c>
-      <c r="L10" s="28" t="n">
+      <c r="L10" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-E10</f>
         <v>-1.6</v>
       </c>
-      <c r="M10" s="28" t="n">
+      <c r="M10" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-F10</f>
         <v>-0.699</v>
       </c>
-      <c r="N10" s="26" t="n">
+      <c r="N10" s="27" t="n">
         <f aca="false">RANK(G10,$G$5:$G$11)</f>
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="C11" s="27" t="n">
+      <c r="A11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="28" t="n">
         <f aca="false">Assumptions!$B$6</f>
         <v>16.99</v>
       </c>
-      <c r="D11" s="28" t="n">
+      <c r="D11" s="29" t="n">
         <f aca="false">Assumptions!$B$6*Assumptions!$B$26</f>
         <v>9.3445</v>
       </c>
-      <c r="E11" s="28" t="n">
+      <c r="E11" s="29" t="n">
         <f aca="false">Assumptions!$B$28</f>
         <v>4</v>
       </c>
-      <c r="F11" s="28" t="n">
+      <c r="F11" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G11" s="29" t="n">
+      <c r="G11" s="30" t="n">
         <f aca="false">C11-D11-E11-F11</f>
         <v>3.6455</v>
       </c>
-      <c r="H11" s="30" t="n">
+      <c r="H11" s="31" t="n">
         <f aca="false">IFERROR(G11/C11,0)</f>
         <v>0.214567392583873</v>
       </c>
-      <c r="I11" s="28" t="n">
+      <c r="I11" s="29" t="n">
         <f aca="false">G11-INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))</f>
         <v>-3.1485</v>
       </c>
-      <c r="J11" s="30" t="n">
+      <c r="J11" s="31" t="n">
         <f aca="false">IFERROR(I11/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))),0)</f>
         <v>-0.463423609066824</v>
       </c>
-      <c r="K11" s="28" t="n">
+      <c r="K11" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-D11</f>
         <v>-2.5485</v>
       </c>
-      <c r="L11" s="28" t="n">
+      <c r="L11" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-E11</f>
         <v>-0.6</v>
       </c>
-      <c r="M11" s="28" t="n">
+      <c r="M11" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$13,$A$5:$A$11,0))-F11</f>
         <v>0</v>
       </c>
-      <c r="N11" s="26" t="n">
+      <c r="N11" s="27" t="n">
         <f aca="false">RANK(G11,$G$5:$G$11)</f>
         <v>4</v>
       </c>
@@ -3993,8 +4010,8 @@
       <c r="N12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>136</v>
+      <c r="A13" s="11" t="s">
+        <v>137</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -4011,8 +4028,8 @@
       <c r="N13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>137</v>
+      <c r="A14" s="16" t="s">
+        <v>138</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -4029,8 +4046,8 @@
       <c r="N14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>138</v>
+      <c r="A15" s="16" t="s">
+        <v>139</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -4047,8 +4064,8 @@
       <c r="N15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
-        <v>139</v>
+      <c r="A16" s="16" t="s">
+        <v>140</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -4065,8 +4082,8 @@
       <c r="N16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
-        <v>140</v>
+      <c r="A17" s="16" t="s">
+        <v>141</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -4083,8 +4100,8 @@
       <c r="N17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>141</v>
+      <c r="A18" s="16" t="s">
+        <v>142</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -4133,8 +4150,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>142</v>
+      <c r="A1" s="13" t="s">
+        <v>143</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -4186,437 +4203,437 @@
       <c r="N3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D4" s="6" t="s">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="C4" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="H4" s="6" t="s">
+      <c r="F4" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="I4" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="L4" s="6" t="s">
+      <c r="J4" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="K4" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="L4" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="N4" s="6" t="s">
-        <v>10</v>
+      <c r="M4" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="C5" s="27" t="n">
+      <c r="A5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="C5" s="28" t="n">
         <f aca="false">Assumptions!$B$8</f>
         <v>4.99</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="29" t="n">
         <f aca="false">(C5-E5)*(1-IF(AND(Assumptions!$B$8&gt;=2.99,Assumptions!$B$8&lt;=9.99),Assumptions!$B$22,Assumptions!$B$23))</f>
         <v>1.407</v>
       </c>
-      <c r="E5" s="28" t="n">
+      <c r="E5" s="29" t="n">
         <f aca="false">IF(AND(Assumptions!$B$8&gt;=2.99,Assumptions!$B$8&lt;=9.99),Assumptions!$B$9*Assumptions!$B$24,0)</f>
         <v>0.3</v>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G5" s="29" t="n">
+      <c r="G5" s="30" t="n">
         <f aca="false">C5-D5-E5-F5</f>
         <v>3.283</v>
       </c>
-      <c r="H5" s="30" t="n">
+      <c r="H5" s="31" t="n">
         <f aca="false">IFERROR(G5/C5,0)</f>
         <v>0.657915831663327</v>
       </c>
-      <c r="I5" s="28" t="n">
+      <c r="I5" s="29" t="n">
         <f aca="false">G5-INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))</f>
         <v>0</v>
       </c>
-      <c r="J5" s="30" t="n">
+      <c r="J5" s="31" t="n">
         <f aca="false">IFERROR(I5/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))),0)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="28" t="n">
+      <c r="K5" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-D5</f>
         <v>0</v>
       </c>
-      <c r="L5" s="28" t="n">
+      <c r="L5" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-E5</f>
         <v>0</v>
       </c>
-      <c r="M5" s="28" t="n">
+      <c r="M5" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-F5</f>
         <v>0</v>
       </c>
-      <c r="N5" s="26" t="n">
+      <c r="N5" s="27" t="n">
         <f aca="false">RANK(G5,$G$5:$G$11)</f>
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="B6" s="26" t="s">
+      <c r="A6" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="B6" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="C6" s="28" t="n">
         <f aca="false">Assumptions!$B$8</f>
         <v>4.99</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="29" t="n">
         <f aca="false">C6*(1-Assumptions!$B$39)</f>
         <v>1.497</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G6" s="29" t="n">
+      <c r="G6" s="30" t="n">
         <f aca="false">C6-D6-E6-F6</f>
         <v>3.493</v>
       </c>
-      <c r="H6" s="30" t="n">
+      <c r="H6" s="31" t="n">
         <f aca="false">IFERROR(G6/C6,0)</f>
         <v>0.7</v>
       </c>
-      <c r="I6" s="28" t="n">
+      <c r="I6" s="29" t="n">
         <f aca="false">G6-INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))</f>
         <v>0.21</v>
       </c>
-      <c r="J6" s="30" t="n">
+      <c r="J6" s="31" t="n">
         <f aca="false">IFERROR(I6/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))),0)</f>
         <v>0.0639658848614071</v>
       </c>
-      <c r="K6" s="28" t="n">
+      <c r="K6" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-D6</f>
         <v>-0.0900000000000001</v>
       </c>
-      <c r="L6" s="28" t="n">
+      <c r="L6" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-E6</f>
         <v>0.3</v>
       </c>
-      <c r="M6" s="28" t="n">
+      <c r="M6" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-F6</f>
         <v>0</v>
       </c>
-      <c r="N6" s="26" t="n">
+      <c r="N6" s="27" t="n">
         <f aca="false">RANK(G6,$G$5:$G$11)</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="C7" s="27" t="n">
+      <c r="A7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="28" t="n">
         <f aca="false">Assumptions!$B$8</f>
         <v>4.99</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="D7" s="29" t="n">
         <f aca="false">C7*(1-Assumptions!$B$33)</f>
         <v>1.497</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F7" s="28" t="n">
+      <c r="F7" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="30" t="n">
         <f aca="false">C7-D7-E7-F7</f>
         <v>3.493</v>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="31" t="n">
         <f aca="false">IFERROR(G7/C7,0)</f>
         <v>0.7</v>
       </c>
-      <c r="I7" s="28" t="n">
+      <c r="I7" s="29" t="n">
         <f aca="false">G7-INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))</f>
         <v>0.21</v>
       </c>
-      <c r="J7" s="30" t="n">
+      <c r="J7" s="31" t="n">
         <f aca="false">IFERROR(I7/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))),0)</f>
         <v>0.0639658848614071</v>
       </c>
-      <c r="K7" s="28" t="n">
+      <c r="K7" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-D7</f>
         <v>-0.0900000000000001</v>
       </c>
-      <c r="L7" s="28" t="n">
+      <c r="L7" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-E7</f>
         <v>0.3</v>
       </c>
-      <c r="M7" s="28" t="n">
+      <c r="M7" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-F7</f>
         <v>0</v>
       </c>
-      <c r="N7" s="26" t="n">
+      <c r="N7" s="27" t="n">
         <f aca="false">RANK(G7,$G$5:$G$11)</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="B8" s="26" t="s">
+      <c r="A8" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="B8" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" s="28" t="n">
         <f aca="false">Assumptions!$B$8</f>
         <v>4.99</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="29" t="n">
         <f aca="false">C8*(1-Assumptions!$B$39)</f>
         <v>1.497</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="29" t="n">
         <f aca="false">(C8-D8)*Assumptions!$B$40</f>
         <v>0.3493</v>
       </c>
-      <c r="G8" s="29" t="n">
+      <c r="G8" s="30" t="n">
         <f aca="false">C8-D8-E8-F8</f>
         <v>3.1437</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="31" t="n">
         <f aca="false">IFERROR(G8/C8,0)</f>
         <v>0.63</v>
       </c>
-      <c r="I8" s="28" t="n">
+      <c r="I8" s="29" t="n">
         <f aca="false">G8-INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))</f>
         <v>-0.1393</v>
       </c>
-      <c r="J8" s="30" t="n">
+      <c r="J8" s="31" t="n">
         <f aca="false">IFERROR(I8/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))),0)</f>
         <v>-0.0424307036247336</v>
       </c>
-      <c r="K8" s="28" t="n">
+      <c r="K8" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-D8</f>
         <v>-0.0900000000000001</v>
       </c>
-      <c r="L8" s="28" t="n">
+      <c r="L8" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-E8</f>
         <v>0.3</v>
       </c>
-      <c r="M8" s="28" t="n">
+      <c r="M8" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-F8</f>
         <v>-0.3493</v>
       </c>
-      <c r="N8" s="26" t="n">
+      <c r="N8" s="27" t="n">
         <f aca="false">RANK(G8,$G$5:$G$11)</f>
         <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="26" t="s">
+      <c r="A9" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="B9" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="C9" s="28" t="n">
         <f aca="false">Assumptions!$B$8</f>
         <v>4.99</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="29" t="n">
         <f aca="false">C9*(1-Assumptions!$B$39)</f>
         <v>1.497</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="29" t="n">
         <f aca="false">(C9-D9)*Assumptions!$B$29</f>
         <v>0.52395</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="30" t="n">
         <f aca="false">C9-D9-E9-F9</f>
         <v>2.96905</v>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="H9" s="31" t="n">
         <f aca="false">IFERROR(G9/C9,0)</f>
         <v>0.595</v>
       </c>
-      <c r="I9" s="28" t="n">
+      <c r="I9" s="29" t="n">
         <f aca="false">G9-INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))</f>
         <v>-0.31395</v>
       </c>
-      <c r="J9" s="30" t="n">
+      <c r="J9" s="31" t="n">
         <f aca="false">IFERROR(I9/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))),0)</f>
         <v>-0.0956289978678039</v>
       </c>
-      <c r="K9" s="28" t="n">
+      <c r="K9" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-D9</f>
         <v>-0.0900000000000001</v>
       </c>
-      <c r="L9" s="28" t="n">
+      <c r="L9" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-E9</f>
         <v>0.3</v>
       </c>
-      <c r="M9" s="28" t="n">
+      <c r="M9" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-F9</f>
         <v>-0.52395</v>
       </c>
-      <c r="N9" s="26" t="n">
+      <c r="N9" s="27" t="n">
         <f aca="false">RANK(G9,$G$5:$G$11)</f>
         <v>6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" s="26" t="s">
+      <c r="A10" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="B10" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="C10" s="28" t="n">
         <f aca="false">Assumptions!$B$8</f>
         <v>4.99</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="29" t="n">
         <f aca="false">C10*(1-Assumptions!$B$39)</f>
         <v>1.497</v>
       </c>
-      <c r="E10" s="28" t="n">
+      <c r="E10" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G10" s="29" t="n">
+      <c r="G10" s="30" t="n">
         <f aca="false">C10-D10-E10-F10</f>
         <v>3.493</v>
       </c>
-      <c r="H10" s="30" t="n">
+      <c r="H10" s="31" t="n">
         <f aca="false">IFERROR(G10/C10,0)</f>
         <v>0.7</v>
       </c>
-      <c r="I10" s="28" t="n">
+      <c r="I10" s="29" t="n">
         <f aca="false">G10-INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))</f>
         <v>0.21</v>
       </c>
-      <c r="J10" s="30" t="n">
+      <c r="J10" s="31" t="n">
         <f aca="false">IFERROR(I10/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))),0)</f>
         <v>0.0639658848614071</v>
       </c>
-      <c r="K10" s="28" t="n">
+      <c r="K10" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-D10</f>
         <v>-0.0900000000000001</v>
       </c>
-      <c r="L10" s="28" t="n">
+      <c r="L10" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-E10</f>
         <v>0.3</v>
       </c>
-      <c r="M10" s="28" t="n">
+      <c r="M10" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-F10</f>
         <v>0</v>
       </c>
-      <c r="N10" s="26" t="n">
+      <c r="N10" s="27" t="n">
         <f aca="false">RANK(G10,$G$5:$G$11)</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="C11" s="27" t="n">
+      <c r="A11" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="28" t="n">
         <f aca="false">Assumptions!$B$8</f>
         <v>4.99</v>
       </c>
-      <c r="D11" s="28" t="n">
+      <c r="D11" s="29" t="n">
         <f aca="false">C11*Assumptions!$B$36</f>
         <v>2.495</v>
       </c>
-      <c r="E11" s="28" t="n">
+      <c r="E11" s="29" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F11" s="28" t="n">
+      <c r="F11" s="29" t="n">
         <f aca="false">(C11-D11)*Assumptions!$B$37</f>
         <v>0.499</v>
       </c>
-      <c r="G11" s="29" t="n">
+      <c r="G11" s="30" t="n">
         <f aca="false">C11-D11-E11-F11</f>
         <v>1.996</v>
       </c>
-      <c r="H11" s="30" t="n">
+      <c r="H11" s="31" t="n">
         <f aca="false">IFERROR(G11/C11,0)</f>
         <v>0.4</v>
       </c>
-      <c r="I11" s="28" t="n">
+      <c r="I11" s="29" t="n">
         <f aca="false">G11-INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))</f>
         <v>-1.287</v>
       </c>
-      <c r="J11" s="30" t="n">
+      <c r="J11" s="31" t="n">
         <f aca="false">IFERROR(I11/ABS(INDEX($G$5:$G$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))),0)</f>
         <v>-0.39201949436491</v>
       </c>
-      <c r="K11" s="28" t="n">
+      <c r="K11" s="29" t="n">
         <f aca="false">INDEX($D$5:$D$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-D11</f>
         <v>-1.088</v>
       </c>
-      <c r="L11" s="28" t="n">
+      <c r="L11" s="29" t="n">
         <f aca="false">INDEX($E$5:$E$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-E11</f>
         <v>0.3</v>
       </c>
-      <c r="M11" s="28" t="n">
+      <c r="M11" s="29" t="n">
         <f aca="false">INDEX($F$5:$F$11,MATCH(Assumptions!$B$14,$A$5:$A$11,0))-F11</f>
         <v>-0.499</v>
       </c>
-      <c r="N11" s="26" t="n">
+      <c r="N11" s="27" t="n">
         <f aca="false">RANK(G11,$G$5:$G$11)</f>
         <v>7</v>
       </c>
@@ -4638,8 +4655,8 @@
       <c r="N12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>161</v>
+      <c r="A13" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -4656,8 +4673,8 @@
       <c r="N13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>162</v>
+      <c r="A14" s="16" t="s">
+        <v>163</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -4674,8 +4691,8 @@
       <c r="N14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>163</v>
+      <c r="A15" s="16" t="s">
+        <v>164</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -4692,8 +4709,8 @@
       <c r="N15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
-        <v>164</v>
+      <c r="A16" s="16" t="s">
+        <v>165</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -4710,8 +4727,8 @@
       <c r="N16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
-        <v>165</v>
+      <c r="A17" s="16" t="s">
+        <v>166</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -4756,8 +4773,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>166</v>
+      <c r="A1" s="13" t="s">
+        <v>167</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -4772,7 +4789,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4799,290 +4816,290 @@
       <c r="K3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="I4" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="J4" s="7" t="s">
         <v>177</v>
       </c>
+      <c r="K4" s="7" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="27" t="n">
+      <c r="A5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G5" s="28" t="n">
+      <c r="G5" s="29" t="n">
         <f aca="false">SUM(B5:F5)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="27" t="n">
+      <c r="H5" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="I5" s="28" t="n">
+      <c r="I5" s="29" t="n">
         <f aca="false">H5*12</f>
         <v>0</v>
       </c>
-      <c r="J5" s="29" t="n">
+      <c r="J5" s="30" t="n">
         <f aca="false">G5+I5</f>
         <v>0</v>
       </c>
-      <c r="K5" s="32" t="s">
-        <v>178</v>
+      <c r="K5" s="33" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="27" t="n">
+      <c r="A6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="28" t="n">
         <f aca="false">Assumptions!$B$42</f>
         <v>125</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="29" t="n">
         <f aca="false">SUM(B6:F6)</f>
         <v>125</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="I6" s="28" t="n">
+      <c r="I6" s="29" t="n">
         <f aca="false">H6*12</f>
         <v>0</v>
       </c>
-      <c r="J6" s="29" t="n">
+      <c r="J6" s="30" t="n">
         <f aca="false">G6+I6</f>
         <v>125</v>
       </c>
-      <c r="K6" s="32" t="s">
-        <v>179</v>
+      <c r="K6" s="33" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="27" t="n">
+      <c r="A7" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="28" t="n">
         <f aca="false">Assumptions!$B$43</f>
         <v>20</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G7" s="28" t="n">
+      <c r="G7" s="29" t="n">
         <f aca="false">SUM(B7:F7)</f>
         <v>20</v>
       </c>
-      <c r="H7" s="27" t="n">
+      <c r="H7" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="I7" s="28" t="n">
+      <c r="I7" s="29" t="n">
         <f aca="false">H7*12</f>
         <v>0</v>
       </c>
-      <c r="J7" s="29" t="n">
+      <c r="J7" s="30" t="n">
         <f aca="false">G7+I7</f>
         <v>20</v>
       </c>
-      <c r="K7" s="32" t="s">
-        <v>180</v>
+      <c r="K7" s="33" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="27" t="n">
+      <c r="A8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="28" t="n">
         <f aca="false">Assumptions!$B$42</f>
         <v>125</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G8" s="28" t="n">
+      <c r="G8" s="29" t="n">
         <f aca="false">SUM(B8:F8)</f>
         <v>125</v>
       </c>
-      <c r="H8" s="27" t="n">
+      <c r="H8" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="I8" s="28" t="n">
+      <c r="I8" s="29" t="n">
         <f aca="false">H8*12</f>
         <v>0</v>
       </c>
-      <c r="J8" s="29" t="n">
+      <c r="J8" s="30" t="n">
         <f aca="false">G8+I8</f>
         <v>125</v>
       </c>
-      <c r="K8" s="32" t="s">
-        <v>181</v>
+      <c r="K8" s="33" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="27" t="n">
+      <c r="A9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="28" t="n">
         <f aca="false">Assumptions!$B$44</f>
         <v>12</v>
       </c>
-      <c r="G9" s="28" t="n">
+      <c r="G9" s="29" t="n">
         <f aca="false">SUM(B9:F9)</f>
         <v>12</v>
       </c>
-      <c r="H9" s="27" t="n">
+      <c r="H9" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="I9" s="28" t="n">
+      <c r="I9" s="29" t="n">
         <f aca="false">H9*12</f>
         <v>0</v>
       </c>
-      <c r="J9" s="29" t="n">
+      <c r="J9" s="30" t="n">
         <f aca="false">G9+I9</f>
         <v>12</v>
       </c>
-      <c r="K9" s="32" t="s">
-        <v>182</v>
+      <c r="K9" s="33" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="27" t="n">
+      <c r="A10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="28" t="n">
         <f aca="false">Assumptions!$B$42</f>
         <v>125</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="28" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="29" t="n">
         <f aca="false">SUM(B10:F10)</f>
         <v>125</v>
       </c>
-      <c r="H10" s="27" t="n">
+      <c r="H10" s="28" t="n">
         <f aca="false">Assumptions!$B$45</f>
         <v>13.99</v>
       </c>
-      <c r="I10" s="28" t="n">
+      <c r="I10" s="29" t="n">
         <f aca="false">H10*12</f>
         <v>167.88</v>
       </c>
-      <c r="J10" s="29" t="n">
+      <c r="J10" s="30" t="n">
         <f aca="false">G10+I10</f>
         <v>292.88</v>
       </c>
-      <c r="K10" s="32" t="s">
-        <v>183</v>
+      <c r="K10" s="33" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -5116,8 +5133,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>184</v>
+      <c r="A1" s="13" t="s">
+        <v>185</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -5172,400 +5189,400 @@
       <c r="O3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="D4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="J4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="I4" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="K4" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="M4" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="N4" s="6" t="s">
+      <c r="L4" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="O4" s="6" t="s">
-        <v>10</v>
+      <c r="M4" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="27" t="n">
+      <c r="A5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="28" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$G$5:$G$11,MATCH(B5,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>6.794</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="28" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$G$5:$G$11,MATCH(C5,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>3.283</v>
       </c>
-      <c r="F5" s="33" t="n">
+      <c r="F5" s="34" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>50</v>
       </c>
-      <c r="G5" s="33" t="n">
+      <c r="G5" s="34" t="n">
         <f aca="false">Assumptions!$B$11</f>
         <v>50</v>
       </c>
-      <c r="H5" s="28" t="n">
+      <c r="H5" s="29" t="n">
         <f aca="false">D5*F5+E5*G5</f>
         <v>503.85</v>
       </c>
-      <c r="I5" s="27" t="n">
+      <c r="I5" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$H$5:$H$10,MATCH(A5,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>0</v>
       </c>
-      <c r="J5" s="28" t="n">
+      <c r="J5" s="29" t="n">
         <f aca="false">H5-I5</f>
         <v>503.85</v>
       </c>
-      <c r="K5" s="28" t="n">
+      <c r="K5" s="29" t="n">
         <f aca="false">J5*12</f>
         <v>6046.2</v>
       </c>
-      <c r="L5" s="27" t="n">
+      <c r="L5" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$G$5:$G$10,MATCH(A5,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>0</v>
       </c>
-      <c r="M5" s="29" t="n">
+      <c r="M5" s="30" t="n">
         <f aca="false">K5-L5</f>
         <v>6046.2</v>
       </c>
-      <c r="N5" s="28" t="n">
+      <c r="N5" s="29" t="n">
         <f aca="false">M5-INDEX($M$5:$M$10,MATCH(Assumptions!$B$15,$A$5:$A$10,0))</f>
         <v>0</v>
       </c>
-      <c r="O5" s="26" t="n">
+      <c r="O5" s="27" t="n">
         <f aca="false">RANK(M5,$M$5:$M$10)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="D6" s="27" t="n">
+      <c r="A6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="28" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$G$5:$G$11,MATCH(B6,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>3.3269375</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="28" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$G$5:$G$11,MATCH(C6,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>2.96905</v>
       </c>
-      <c r="F6" s="33" t="n">
+      <c r="F6" s="34" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>50</v>
       </c>
-      <c r="G6" s="33" t="n">
+      <c r="G6" s="34" t="n">
         <f aca="false">Assumptions!$B$11</f>
         <v>50</v>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="H6" s="29" t="n">
         <f aca="false">D6*F6+E6*G6</f>
         <v>314.799375</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$H$5:$H$10,MATCH(A6,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>0</v>
       </c>
-      <c r="J6" s="28" t="n">
+      <c r="J6" s="29" t="n">
         <f aca="false">H6-I6</f>
         <v>314.799375</v>
       </c>
-      <c r="K6" s="28" t="n">
+      <c r="K6" s="29" t="n">
         <f aca="false">J6*12</f>
         <v>3777.5925</v>
       </c>
-      <c r="L6" s="27" t="n">
+      <c r="L6" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$G$5:$G$10,MATCH(A6,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>125</v>
       </c>
-      <c r="M6" s="29" t="n">
+      <c r="M6" s="30" t="n">
         <f aca="false">K6-L6</f>
         <v>3652.5925</v>
       </c>
-      <c r="N6" s="28" t="n">
+      <c r="N6" s="29" t="n">
         <f aca="false">M6-INDEX($M$5:$M$10,MATCH(Assumptions!$B$15,$A$5:$A$10,0))</f>
         <v>-2393.6075</v>
       </c>
-      <c r="O6" s="26" t="n">
+      <c r="O6" s="27" t="n">
         <f aca="false">RANK(M6,$M$5:$M$10)</f>
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="27" t="n">
+      <c r="A7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="28" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$G$5:$G$11,MATCH(B7,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>5.8445</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="28" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$G$5:$G$11,MATCH(C7,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>3.493</v>
       </c>
-      <c r="F7" s="33" t="n">
+      <c r="F7" s="34" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>50</v>
       </c>
-      <c r="G7" s="33" t="n">
+      <c r="G7" s="34" t="n">
         <f aca="false">Assumptions!$B$11</f>
         <v>50</v>
       </c>
-      <c r="H7" s="28" t="n">
+      <c r="H7" s="29" t="n">
         <f aca="false">D7*F7+E7*G7</f>
         <v>466.875</v>
       </c>
-      <c r="I7" s="27" t="n">
+      <c r="I7" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$H$5:$H$10,MATCH(A7,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>0</v>
       </c>
-      <c r="J7" s="28" t="n">
+      <c r="J7" s="29" t="n">
         <f aca="false">H7-I7</f>
         <v>466.875</v>
       </c>
-      <c r="K7" s="28" t="n">
+      <c r="K7" s="29" t="n">
         <f aca="false">J7*12</f>
         <v>5602.5</v>
       </c>
-      <c r="L7" s="27" t="n">
+      <c r="L7" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$G$5:$G$10,MATCH(A7,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>125</v>
       </c>
-      <c r="M7" s="29" t="n">
+      <c r="M7" s="30" t="n">
         <f aca="false">K7-L7</f>
         <v>5477.5</v>
       </c>
-      <c r="N7" s="28" t="n">
+      <c r="N7" s="29" t="n">
         <f aca="false">M7-INDEX($M$5:$M$10,MATCH(Assumptions!$B$15,$A$5:$A$10,0))</f>
         <v>-568.699999999999</v>
       </c>
-      <c r="O7" s="26" t="n">
+      <c r="O7" s="27" t="n">
         <f aca="false">RANK(M7,$M$5:$M$10)</f>
         <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="D8" s="27" t="n">
+      <c r="A8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D8" s="28" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$G$5:$G$11,MATCH(B8,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>2.796</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="28" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$G$5:$G$11,MATCH(C8,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>1.996</v>
       </c>
-      <c r="F8" s="33" t="n">
+      <c r="F8" s="34" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>50</v>
       </c>
-      <c r="G8" s="33" t="n">
+      <c r="G8" s="34" t="n">
         <f aca="false">Assumptions!$B$11</f>
         <v>50</v>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="29" t="n">
         <f aca="false">D8*F8+E8*G8</f>
         <v>239.6</v>
       </c>
-      <c r="I8" s="27" t="n">
+      <c r="I8" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$H$5:$H$10,MATCH(A8,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>0</v>
       </c>
-      <c r="J8" s="28" t="n">
+      <c r="J8" s="29" t="n">
         <f aca="false">H8-I8</f>
         <v>239.6</v>
       </c>
-      <c r="K8" s="28" t="n">
+      <c r="K8" s="29" t="n">
         <f aca="false">J8*12</f>
         <v>2875.2</v>
       </c>
-      <c r="L8" s="27" t="n">
+      <c r="L8" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$G$5:$G$10,MATCH(A8,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>12</v>
       </c>
-      <c r="M8" s="29" t="n">
+      <c r="M8" s="30" t="n">
         <f aca="false">K8-L8</f>
         <v>2863.2</v>
       </c>
-      <c r="N8" s="28" t="n">
+      <c r="N8" s="29" t="n">
         <f aca="false">M8-INDEX($M$5:$M$10,MATCH(Assumptions!$B$15,$A$5:$A$10,0))</f>
         <v>-3183</v>
       </c>
-      <c r="O8" s="26" t="n">
+      <c r="O8" s="27" t="n">
         <f aca="false">RANK(M8,$M$5:$M$10)</f>
         <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="D9" s="27" t="n">
+      <c r="A9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" s="28" t="n">
         <f aca="false">INDEX('Print Unit Econ'!$G$5:$G$11,MATCH(B9,'Print Unit Econ'!$A$5:$A$11,0))</f>
         <v>3.6455</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="28" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$G$5:$G$11,MATCH(C9,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>3.493</v>
       </c>
-      <c r="F9" s="33" t="n">
+      <c r="F9" s="34" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>50</v>
       </c>
-      <c r="G9" s="33" t="n">
+      <c r="G9" s="34" t="n">
         <f aca="false">Assumptions!$B$11</f>
         <v>50</v>
       </c>
-      <c r="H9" s="28" t="n">
+      <c r="H9" s="29" t="n">
         <f aca="false">D9*F9+E9*G9</f>
         <v>356.925</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$H$5:$H$10,MATCH(A9,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>13.99</v>
       </c>
-      <c r="J9" s="28" t="n">
+      <c r="J9" s="29" t="n">
         <f aca="false">H9-I9</f>
         <v>342.935</v>
       </c>
-      <c r="K9" s="28" t="n">
+      <c r="K9" s="29" t="n">
         <f aca="false">J9*12</f>
         <v>4115.22</v>
       </c>
-      <c r="L9" s="27" t="n">
+      <c r="L9" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$G$5:$G$10,MATCH(A9,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>125</v>
       </c>
-      <c r="M9" s="29" t="n">
+      <c r="M9" s="30" t="n">
         <f aca="false">K9-L9</f>
         <v>3990.22</v>
       </c>
-      <c r="N9" s="28" t="n">
+      <c r="N9" s="29" t="n">
         <f aca="false">M9-INDEX($M$5:$M$10,MATCH(Assumptions!$B$15,$A$5:$A$10,0))</f>
         <v>-2055.98</v>
       </c>
-      <c r="O9" s="26" t="n">
+      <c r="O9" s="27" t="n">
         <f aca="false">RANK(M9,$M$5:$M$10)</f>
         <v>3</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>194</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="D10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="27" t="n">
+      <c r="A10" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="28" t="n">
         <f aca="false">INDEX('Ebook Unit Econ'!$G$5:$G$11,MATCH(C10,'Ebook Unit Econ'!$A$5:$A$11,0))</f>
         <v>3.1437</v>
       </c>
-      <c r="F10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="33" t="n">
+      <c r="F10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="34" t="n">
         <f aca="false">Assumptions!$B$11</f>
         <v>50</v>
       </c>
-      <c r="H10" s="28" t="n">
+      <c r="H10" s="29" t="n">
         <f aca="false">D10*F10+E10*G10</f>
         <v>157.185</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$H$5:$H$10,MATCH(A10,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>0</v>
       </c>
-      <c r="J10" s="28" t="n">
+      <c r="J10" s="29" t="n">
         <f aca="false">H10-I10</f>
         <v>157.185</v>
       </c>
-      <c r="K10" s="28" t="n">
+      <c r="K10" s="29" t="n">
         <f aca="false">J10*12</f>
         <v>1886.22</v>
       </c>
-      <c r="L10" s="27" t="n">
+      <c r="L10" s="28" t="n">
         <f aca="false">INDEX('Fixed Costs'!$G$5:$G$10,MATCH(A10,'Fixed Costs'!$A$5:$A$10,0))</f>
         <v>20</v>
       </c>
-      <c r="M10" s="29" t="n">
+      <c r="M10" s="30" t="n">
         <f aca="false">K10-L10</f>
         <v>1866.22</v>
       </c>
-      <c r="N10" s="28" t="n">
+      <c r="N10" s="29" t="n">
         <f aca="false">M10-INDEX($M$5:$M$10,MATCH(Assumptions!$B$15,$A$5:$A$10,0))</f>
         <v>-4179.98</v>
       </c>
-      <c r="O10" s="26" t="n">
+      <c r="O10" s="27" t="n">
         <f aca="false">RANK(M10,$M$5:$M$10)</f>
         <v>6</v>
       </c>
@@ -5588,8 +5605,8 @@
       <c r="O11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>161</v>
+      <c r="A12" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -5607,8 +5624,8 @@
       <c r="O12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
-        <v>195</v>
+      <c r="A13" s="16" t="s">
+        <v>196</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -5626,8 +5643,8 @@
       <c r="O13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>196</v>
+      <c r="A14" s="16" t="s">
+        <v>197</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -5645,8 +5662,8 @@
       <c r="O14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>197</v>
+      <c r="A15" s="16" t="s">
+        <v>198</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -5687,8 +5704,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>198</v>
+      <c r="A1" s="13" t="s">
+        <v>199</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -5699,7 +5716,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -5718,221 +5735,221 @@
       <c r="G3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>205</v>
       </c>
+      <c r="G4" s="7" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="B5" s="19" t="n">
+      <c r="A5" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B5" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="20" t="n">
         <v>250</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="20" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="34" t="n">
+      <c r="A6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="35" t="n">
         <f aca="false">B$5*('Monthly Scenario'!$D$5+'Monthly Scenario'!$E$5)-'Monthly Scenario'!$I$5</f>
         <v>100.77</v>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="35" t="n">
         <f aca="false">C$5*('Monthly Scenario'!$D$5+'Monthly Scenario'!$E$5)-'Monthly Scenario'!$I$5</f>
         <v>251.925</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="35" t="n">
         <f aca="false">D$5*('Monthly Scenario'!$D$5+'Monthly Scenario'!$E$5)-'Monthly Scenario'!$I$5</f>
         <v>503.85</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="35" t="n">
         <f aca="false">E$5*('Monthly Scenario'!$D$5+'Monthly Scenario'!$E$5)-'Monthly Scenario'!$I$5</f>
         <v>1007.7</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="35" t="n">
         <f aca="false">F$5*('Monthly Scenario'!$D$5+'Monthly Scenario'!$E$5)-'Monthly Scenario'!$I$5</f>
         <v>2519.25</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G6" s="35" t="n">
         <f aca="false">G$5*('Monthly Scenario'!$D$5+'Monthly Scenario'!$E$5)-'Monthly Scenario'!$I$5</f>
         <v>5038.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="34" t="n">
+      <c r="A7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="35" t="n">
         <f aca="false">B$5*('Monthly Scenario'!$D$6+'Monthly Scenario'!$E$6)-'Monthly Scenario'!$I$6</f>
         <v>62.959875</v>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="C7" s="35" t="n">
         <f aca="false">C$5*('Monthly Scenario'!$D$6+'Monthly Scenario'!$E$6)-'Monthly Scenario'!$I$6</f>
         <v>157.3996875</v>
       </c>
-      <c r="D7" s="34" t="n">
+      <c r="D7" s="35" t="n">
         <f aca="false">D$5*('Monthly Scenario'!$D$6+'Monthly Scenario'!$E$6)-'Monthly Scenario'!$I$6</f>
         <v>314.799375</v>
       </c>
-      <c r="E7" s="34" t="n">
+      <c r="E7" s="35" t="n">
         <f aca="false">E$5*('Monthly Scenario'!$D$6+'Monthly Scenario'!$E$6)-'Monthly Scenario'!$I$6</f>
         <v>629.59875</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="35" t="n">
         <f aca="false">F$5*('Monthly Scenario'!$D$6+'Monthly Scenario'!$E$6)-'Monthly Scenario'!$I$6</f>
         <v>1573.996875</v>
       </c>
-      <c r="G7" s="34" t="n">
+      <c r="G7" s="35" t="n">
         <f aca="false">G$5*('Monthly Scenario'!$D$6+'Monthly Scenario'!$E$6)-'Monthly Scenario'!$I$6</f>
         <v>3147.99375</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="34" t="n">
+      <c r="A8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="35" t="n">
         <f aca="false">B$5*('Monthly Scenario'!$D$7+'Monthly Scenario'!$E$7)-'Monthly Scenario'!$I$7</f>
         <v>93.375</v>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="35" t="n">
         <f aca="false">C$5*('Monthly Scenario'!$D$7+'Monthly Scenario'!$E$7)-'Monthly Scenario'!$I$7</f>
         <v>233.4375</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="35" t="n">
         <f aca="false">D$5*('Monthly Scenario'!$D$7+'Monthly Scenario'!$E$7)-'Monthly Scenario'!$I$7</f>
         <v>466.875</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="35" t="n">
         <f aca="false">E$5*('Monthly Scenario'!$D$7+'Monthly Scenario'!$E$7)-'Monthly Scenario'!$I$7</f>
         <v>933.75</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="35" t="n">
         <f aca="false">F$5*('Monthly Scenario'!$D$7+'Monthly Scenario'!$E$7)-'Monthly Scenario'!$I$7</f>
         <v>2334.375</v>
       </c>
-      <c r="G8" s="34" t="n">
+      <c r="G8" s="35" t="n">
         <f aca="false">G$5*('Monthly Scenario'!$D$7+'Monthly Scenario'!$E$7)-'Monthly Scenario'!$I$7</f>
         <v>4668.75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="34" t="n">
+      <c r="A9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="35" t="n">
         <f aca="false">B$5*('Monthly Scenario'!$D$8+'Monthly Scenario'!$E$8)-'Monthly Scenario'!$I$8</f>
         <v>47.92</v>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="C9" s="35" t="n">
         <f aca="false">C$5*('Monthly Scenario'!$D$8+'Monthly Scenario'!$E$8)-'Monthly Scenario'!$I$8</f>
         <v>119.8</v>
       </c>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="35" t="n">
         <f aca="false">D$5*('Monthly Scenario'!$D$8+'Monthly Scenario'!$E$8)-'Monthly Scenario'!$I$8</f>
         <v>239.6</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="35" t="n">
         <f aca="false">E$5*('Monthly Scenario'!$D$8+'Monthly Scenario'!$E$8)-'Monthly Scenario'!$I$8</f>
         <v>479.2</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="35" t="n">
         <f aca="false">F$5*('Monthly Scenario'!$D$8+'Monthly Scenario'!$E$8)-'Monthly Scenario'!$I$8</f>
         <v>1198</v>
       </c>
-      <c r="G9" s="34" t="n">
+      <c r="G9" s="35" t="n">
         <f aca="false">G$5*('Monthly Scenario'!$D$8+'Monthly Scenario'!$E$8)-'Monthly Scenario'!$I$8</f>
         <v>2396</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="34" t="n">
+      <c r="A10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="35" t="n">
         <f aca="false">B$5*('Monthly Scenario'!$D$9+'Monthly Scenario'!$E$9)-'Monthly Scenario'!$I$9</f>
         <v>57.395</v>
       </c>
-      <c r="C10" s="34" t="n">
+      <c r="C10" s="35" t="n">
         <f aca="false">C$5*('Monthly Scenario'!$D$9+'Monthly Scenario'!$E$9)-'Monthly Scenario'!$I$9</f>
         <v>164.4725</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="35" t="n">
         <f aca="false">D$5*('Monthly Scenario'!$D$9+'Monthly Scenario'!$E$9)-'Monthly Scenario'!$I$9</f>
         <v>342.935</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="35" t="n">
         <f aca="false">E$5*('Monthly Scenario'!$D$9+'Monthly Scenario'!$E$9)-'Monthly Scenario'!$I$9</f>
         <v>699.86</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="35" t="n">
         <f aca="false">F$5*('Monthly Scenario'!$D$9+'Monthly Scenario'!$E$9)-'Monthly Scenario'!$I$9</f>
         <v>1770.635</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G10" s="35" t="n">
         <f aca="false">G$5*('Monthly Scenario'!$D$9+'Monthly Scenario'!$E$9)-'Monthly Scenario'!$I$9</f>
         <v>3555.26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="34" t="n">
+      <c r="A11" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="35" t="n">
         <f aca="false">B$5*('Monthly Scenario'!$D$10+'Monthly Scenario'!$E$10)-'Monthly Scenario'!$I$10</f>
         <v>31.437</v>
       </c>
-      <c r="C11" s="34" t="n">
+      <c r="C11" s="35" t="n">
         <f aca="false">C$5*('Monthly Scenario'!$D$10+'Monthly Scenario'!$E$10)-'Monthly Scenario'!$I$10</f>
         <v>78.5925</v>
       </c>
-      <c r="D11" s="34" t="n">
+      <c r="D11" s="35" t="n">
         <f aca="false">D$5*('Monthly Scenario'!$D$10+'Monthly Scenario'!$E$10)-'Monthly Scenario'!$I$10</f>
         <v>157.185</v>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="35" t="n">
         <f aca="false">E$5*('Monthly Scenario'!$D$10+'Monthly Scenario'!$E$10)-'Monthly Scenario'!$I$10</f>
         <v>314.37</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="35" t="n">
         <f aca="false">F$5*('Monthly Scenario'!$D$10+'Monthly Scenario'!$E$10)-'Monthly Scenario'!$I$10</f>
         <v>785.925</v>
       </c>
-      <c r="G11" s="34" t="n">
+      <c r="G11" s="35" t="n">
         <f aca="false">G$5*('Monthly Scenario'!$D$10+'Monthly Scenario'!$E$10)-'Monthly Scenario'!$I$10</f>
         <v>1571.85</v>
       </c>
@@ -5947,8 +5964,8 @@
       <c r="G12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>207</v>
+      <c r="A13" s="14" t="s">
+        <v>208</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -5958,13 +5975,13 @@
       <c r="G13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="35" t="s">
-        <v>208</v>
-      </c>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36" t="n">
+      <c r="A14" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="37" t="n">
         <f aca="false">IFERROR('Monthly Scenario'!I9/(('Monthly Scenario'!D9+'Monthly Scenario'!E9)-('Monthly Scenario'!D6+'Monthly Scenario'!E6)),"n/a")</f>
         <v>16.6050948798979</v>
       </c>
@@ -5972,13 +5989,13 @@
       <c r="G14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="35" t="s">
-        <v>209</v>
-      </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36" t="n">
+      <c r="A15" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="B15" s="36"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="37" t="n">
         <f aca="false">IFERROR('Monthly Scenario'!I9/('Monthly Scenario'!E9-'Monthly Scenario'!E10),"n/a")</f>
         <v>40.051531634698</v>
       </c>
@@ -6014,8 +6031,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>210</v>
+      <c r="A1" s="13" t="s">
+        <v>211</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -6026,157 +6043,157 @@
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>213</v>
       </c>
+      <c r="C3" s="7" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>214</v>
-      </c>
-      <c r="B4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>215</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="B4" s="16" t="s">
         <v>216</v>
       </c>
+      <c r="C4" s="38" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>217</v>
-      </c>
-      <c r="B5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>218</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="B5" s="16" t="s">
         <v>219</v>
       </c>
+      <c r="C5" s="38" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>220</v>
-      </c>
-      <c r="B6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="B6" s="16" t="s">
         <v>222</v>
       </c>
+      <c r="C6" s="38" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="B7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="B7" s="16" t="s">
         <v>225</v>
       </c>
+      <c r="C7" s="38" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>226</v>
-      </c>
-      <c r="B8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="B8" s="16" t="s">
         <v>228</v>
       </c>
+      <c r="C8" s="38" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>229</v>
-      </c>
-      <c r="B9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>230</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="B9" s="16" t="s">
         <v>231</v>
       </c>
+      <c r="C9" s="38" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>232</v>
-      </c>
-      <c r="C10" s="37" t="s">
+      <c r="A10" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="B10" s="16" t="s">
         <v>233</v>
       </c>
+      <c r="C10" s="38" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
-        <v>234</v>
-      </c>
-      <c r="B11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="C11" s="37" t="s">
+      <c r="B11" s="16" t="s">
         <v>236</v>
       </c>
+      <c r="C11" s="38" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>237</v>
-      </c>
-      <c r="B12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>238</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="B12" s="16" t="s">
         <v>239</v>
       </c>
+      <c r="C12" s="38" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
-        <v>240</v>
-      </c>
-      <c r="B13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="C13" s="37" t="s">
+      <c r="B13" s="16" t="s">
         <v>242</v>
       </c>
+      <c r="C13" s="38" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>243</v>
-      </c>
-      <c r="B14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>244</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="B14" s="16" t="s">
         <v>245</v>
       </c>
+      <c r="C14" s="38" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>246</v>
-      </c>
-      <c r="B15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>247</v>
       </c>
-      <c r="C15" s="37" t="s">
+      <c r="B15" s="16" t="s">
         <v>248</v>
       </c>
+      <c r="C15" s="38" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
-        <v>249</v>
-      </c>
-      <c r="B16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>250</v>
       </c>
-      <c r="C16" s="37" t="s">
+      <c r="B16" s="16" t="s">
         <v>251</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6186,7 +6203,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>

</xml_diff>

<commit_message>
Title Case for all titles and subheadings; sources card moves before recommendations
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018GGaLYafumZWSzZZvAq2bQ
</commit_message>
<xml_diff>
--- a/workbook/IP_Distribution_Cost_Variance_Model.xlsx
+++ b/workbook/IP_Distribution_Cost_Variance_Model.xlsx
@@ -612,7 +612,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -716,7 +716,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -806,7 +806,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -914,7 +914,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1024,7 +1024,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1114,7 +1114,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1222,7 +1222,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1332,7 +1332,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1422,7 +1422,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>

</xml_diff>